<commit_message>
feat: implement layer-based depth pruning and add sensitivity analysis support for YOLOv5 and RT-DETR models
</commit_message>
<xml_diff>
--- a/benchmarks/benchmark_results_rtdetr.xlsx
+++ b/benchmarks/benchmark_results_rtdetr.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Model Name</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Total Latency (ms/img)</t>
   </si>
   <si>
+    <t>FPS</t>
+  </si>
+  <si>
     <t>Baseline</t>
   </si>
   <si>
@@ -58,7 +61,7 @@
     <t>PekingU/rtdetr_r18vd</t>
   </si>
   <si>
-    <t>rtdetr-pruned.pt</t>
+    <t>weights/rtdetr-pruned.pt</t>
   </si>
 </sst>
 </file>
@@ -390,10 +393,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -427,13 +430,16 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>20174608</v>
@@ -442,60 +448,66 @@
         <v>61.243</v>
       </c>
       <c r="E2">
-        <v>0.6516</v>
+        <v>0.6496</v>
       </c>
       <c r="F2">
-        <v>0.6938</v>
+        <v>0.6864</v>
       </c>
       <c r="G2">
-        <v>0.6516</v>
+        <v>0.6496</v>
       </c>
       <c r="H2">
-        <v>0.4844</v>
+        <v>0.4744</v>
       </c>
       <c r="I2">
-        <v>446</v>
+        <v>492.13</v>
       </c>
       <c r="J2">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="K2">
-        <v>446.23</v>
+        <v>492.41</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3">
-        <v>16346740</v>
+        <v>19035420</v>
       </c>
       <c r="D3">
-        <v>53.588</v>
+        <v>59.01</v>
       </c>
       <c r="E3">
-        <v>0.3782</v>
+        <v>0.0945</v>
       </c>
       <c r="F3">
-        <v>0.4998</v>
+        <v>0.2492</v>
       </c>
       <c r="G3">
-        <v>0.3782</v>
+        <v>0.0945</v>
       </c>
       <c r="H3">
-        <v>0.2665</v>
+        <v>0.0612</v>
       </c>
       <c r="I3">
-        <v>388.45</v>
+        <v>433.1</v>
       </c>
       <c r="J3">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="K3">
-        <v>388.69</v>
+        <v>433.35</v>
+      </c>
+      <c r="L3">
+        <v>2.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>